<commit_message>
EP007 y EP008: plantillas comprobadas en Google Sheets (nota en el README); EP008 sin #N/A en la hoja vacía y con la columna A más ancha
</commit_message>
<xml_diff>
--- a/EP008/plantilla_comprobar_cambios.xlsx
+++ b/EP008/plantilla_comprobar_cambios.xlsx
@@ -52,9 +52,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -103,7 +103,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>MAXIFS(F6:F205,C6:C205,"*recio*")</f>
+        <f>IF(COUNTIFS(C6:C205,"*recio*",F6:F205,"&gt;0")=0,"",MAXIFS(F6:F205,C6:C205,"*recio*"))</f>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -111,7 +111,7 @@
         </is>
       </c>
       <c r="D4" t="str">
-        <f>INDEX(A6:A205,MATCH(1,INDEX((F6:F205=B4)*ISNUMBER(SEARCH("recio",C6:C205)),0),0))</f>
+        <f>IFERROR(INDEX(A6:A205,MATCH(1,INDEX((F6:F205=B4)*ISNUMBER(SEARCH("recio",C6:C205)),0),0)),"")</f>
       </c>
     </row>
     <row r="5">
@@ -1758,9 +1758,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>MAXIFS(F6:F205,C6:C205,"*recio*")</f>
+        <f>IF(COUNTIFS(C6:C205,"*recio*",F6:F205,"&gt;0")=0,"",MAXIFS(F6:F205,C6:C205,"*recio*"))</f>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="D4" t="str">
-        <f>INDEX(A6:A205,MATCH(1,INDEX((F6:F205=B4)*ISNUMBER(SEARCH("recio",C6:C205)),0),0))</f>
+        <f>IFERROR(INDEX(A6:A205,MATCH(1,INDEX((F6:F205=B4)*ISNUMBER(SEARCH("recio",C6:C205)),0),0)),"")</f>
       </c>
     </row>
     <row r="5">

</xml_diff>